<commit_message>
Updated employee data and fixed banner text
</commit_message>
<xml_diff>
--- a/sample_data.xlsx
+++ b/sample_data.xlsx
@@ -448,16 +448,16 @@
         <v>EMP001</v>
       </c>
       <c r="B2" t="str">
-        <v>Rahul Sharma</v>
+        <v>Guru Charan</v>
       </c>
       <c r="C2" t="str">
         <v>Engineering</v>
       </c>
       <c r="D2" t="str">
-        <v>Software Engineer</v>
+        <v>Senior Developer</v>
       </c>
       <c r="E2">
-        <v>85000</v>
+        <v>125000</v>
       </c>
       <c r="F2" t="str">
         <v>Bangalore</v>
@@ -480,16 +480,16 @@
         <v>EMP002</v>
       </c>
       <c r="B3" t="str">
-        <v>Priya Patel</v>
+        <v>Guru Dayal</v>
       </c>
       <c r="C3" t="str">
         <v>Marketing</v>
       </c>
       <c r="D3" t="str">
-        <v>Marketing Manager</v>
+        <v>Senior Developer</v>
       </c>
       <c r="E3">
-        <v>92000</v>
+        <v>120000</v>
       </c>
       <c r="F3" t="str">
         <v>Mumbai</v>
@@ -512,13 +512,13 @@
         <v>EMP003</v>
       </c>
       <c r="B4" t="str">
-        <v>Amit Kumar</v>
+        <v>Sai Rajesh</v>
       </c>
       <c r="C4" t="str">
         <v>Engineering</v>
       </c>
       <c r="D4" t="str">
-        <v>Senior Developer</v>
+        <v>Developer</v>
       </c>
       <c r="E4">
         <v>110000</v>

</xml_diff>